<commit_message>
Parte pequeño sin columnas N y O; P.H. BALSA en el parte grande; fuera lo de reciclada
- Control de aportes: se quitan las columnas N y O y la de trazabilidad se ensancha, como la hoja nueva.
- Control de riegos: la fila E.C. RECICLADA pasa a P.H. BALSA.
- En la app ya no se apunta CE reciclada, incremento reciclada ni m³ reciclada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016whyeuvWmXjpnmK3jvZ2dv
</commit_message>
<xml_diff>
--- a/fuente/plantilla2/parte.xlsx
+++ b/fuente/plantilla2/parte.xlsx
@@ -2553,10 +2553,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="14" max="14" width="19" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="15.75" thickBot="1">
+    <row r="1" spans="1:19" ht="15.75" thickBot="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2576,10 +2579,8 @@
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-    </row>
-    <row r="2" spans="1:21">
+    </row>
+    <row r="2" spans="1:19">
       <c r="A2" s="2"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2600,11 +2601,9 @@
       <c r="P2" s="6"/>
       <c r="Q2" s="6"/>
       <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="7"/>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" thickBot="1">
+      <c r="S2" s="7"/>
+    </row>
+    <row r="3" spans="1:19" ht="15.75" thickBot="1">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -2623,11 +2622,9 @@
       <c r="P3" s="12"/>
       <c r="Q3" s="12"/>
       <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="13"/>
-    </row>
-    <row r="4" spans="1:21">
+      <c r="S3" s="13"/>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4" s="8"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -2648,11 +2645,9 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="7"/>
-    </row>
-    <row r="5" spans="1:21" ht="15.75" thickBot="1">
+      <c r="S4" s="7"/>
+    </row>
+    <row r="5" spans="1:19" ht="15.75" thickBot="1">
       <c r="A5" s="14"/>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -2671,11 +2666,9 @@
       <c r="P5" s="18"/>
       <c r="Q5" s="18"/>
       <c r="R5" s="18"/>
-      <c r="S5" s="18"/>
-      <c r="T5" s="18"/>
-      <c r="U5" s="19"/>
-    </row>
-    <row r="6" spans="1:21" ht="15.75" thickBot="1">
+      <c r="S5" s="19"/>
+    </row>
+    <row r="6" spans="1:19" ht="15.75" thickBot="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -2695,10 +2688,8 @@
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
-      <c r="T6" s="1"/>
-      <c r="U6" s="1"/>
-    </row>
-    <row r="7" spans="1:21" ht="19.5" thickTop="1" thickBot="1">
+    </row>
+    <row r="7" spans="1:19" ht="19.5" thickTop="1" thickBot="1">
       <c r="A7" s="20" t="s">
         <v>2</v>
       </c>
@@ -2719,11 +2710,9 @@
       <c r="P7" s="21"/>
       <c r="Q7" s="21"/>
       <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="21"/>
-      <c r="U7" s="22"/>
-    </row>
-    <row r="8" spans="1:21" ht="17.25" thickTop="1" thickBot="1">
+      <c r="S7" s="22"/>
+    </row>
+    <row r="8" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A8" s="23" t="s">
         <v>3</v>
       </c>
@@ -2739,18 +2728,16 @@
       <c r="K8" s="27"/>
       <c r="L8" s="27"/>
       <c r="M8" s="27"/>
-      <c r="N8" s="28"/>
-      <c r="O8" s="29"/>
-      <c r="P8" s="23" t="s">
+      <c r="N8" s="23" t="s">
         <v>4</v>
       </c>
+      <c r="O8" s="30"/>
+      <c r="P8" s="30"/>
       <c r="Q8" s="30"/>
       <c r="R8" s="30"/>
-      <c r="S8" s="30"/>
-      <c r="T8" s="30"/>
-      <c r="U8" s="31"/>
-    </row>
-    <row r="9" spans="1:21" ht="16.5" thickTop="1" thickBot="1">
+      <c r="S8" s="31"/>
+    </row>
+    <row r="9" spans="1:19" ht="16.5" thickTop="1" thickBot="1">
       <c r="A9" s="32" t="s">
         <v>5</v>
       </c>
@@ -2770,16 +2757,14 @@
       <c r="K9" s="37"/>
       <c r="L9" s="37"/>
       <c r="M9" s="38"/>
-      <c r="N9" s="39"/>
-      <c r="O9" s="40"/>
-      <c r="P9" s="41"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="42"/>
+      <c r="P9" s="42"/>
       <c r="Q9" s="42"/>
       <c r="R9" s="42"/>
-      <c r="S9" s="42"/>
-      <c r="T9" s="42"/>
-      <c r="U9" s="43"/>
-    </row>
-    <row r="10" spans="1:21" ht="16.5" thickTop="1" thickBot="1">
+      <c r="S9" s="43"/>
+    </row>
+    <row r="10" spans="1:19" ht="16.5" thickTop="1" thickBot="1">
       <c r="A10" s="44" t="s">
         <v>8</v>
       </c>
@@ -2805,24 +2790,22 @@
       <c r="M10" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="N10" s="51"/>
-      <c r="O10" s="51"/>
-      <c r="P10" s="52" t="s">
+      <c r="N10" s="52" t="s">
         <v>14</v>
       </c>
+      <c r="O10" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="P10" s="54"/>
       <c r="Q10" s="53" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R10" s="54"/>
-      <c r="S10" s="53" t="s">
-        <v>16</v>
-      </c>
-      <c r="T10" s="54"/>
-      <c r="U10" s="55" t="s">
+      <c r="S10" s="55" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="17.25" thickTop="1" thickBot="1">
+    <row r="11" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A11" s="56" t="s">
         <v>18</v>
       </c>
@@ -2840,18 +2823,16 @@
       <c r="K11" s="64"/>
       <c r="L11" s="64"/>
       <c r="M11" s="65"/>
-      <c r="N11" s="66"/>
-      <c r="O11" s="66"/>
-      <c r="P11" s="67" t="s">
+      <c r="N11" s="67" t="s">
         <v>20</v>
       </c>
+      <c r="O11" s="68"/>
+      <c r="P11" s="69"/>
       <c r="Q11" s="68"/>
       <c r="R11" s="69"/>
-      <c r="S11" s="68"/>
-      <c r="T11" s="69"/>
-      <c r="U11" s="70"/>
-    </row>
-    <row r="12" spans="1:21" ht="15.75">
+      <c r="S11" s="70"/>
+    </row>
+    <row r="12" spans="1:19" ht="15.75">
       <c r="A12" s="71" t="s">
         <v>21</v>
       </c>
@@ -2869,16 +2850,14 @@
       <c r="K12" s="79"/>
       <c r="L12" s="79"/>
       <c r="M12" s="80"/>
-      <c r="N12" s="66"/>
-      <c r="O12" s="66"/>
-      <c r="P12" s="81"/>
+      <c r="N12" s="81"/>
+      <c r="O12" s="82"/>
+      <c r="P12" s="83"/>
       <c r="Q12" s="82"/>
       <c r="R12" s="83"/>
-      <c r="S12" s="82"/>
-      <c r="T12" s="83"/>
-      <c r="U12" s="84"/>
-    </row>
-    <row r="13" spans="1:21" ht="15.75">
+      <c r="S12" s="84"/>
+    </row>
+    <row r="13" spans="1:19" ht="15.75">
       <c r="A13" s="71" t="s">
         <v>23</v>
       </c>
@@ -2896,16 +2875,14 @@
       <c r="K13" s="79"/>
       <c r="L13" s="79"/>
       <c r="M13" s="80"/>
-      <c r="N13" s="66"/>
-      <c r="O13" s="66"/>
-      <c r="P13" s="81"/>
+      <c r="N13" s="81"/>
+      <c r="O13" s="82"/>
+      <c r="P13" s="83"/>
       <c r="Q13" s="82"/>
       <c r="R13" s="83"/>
-      <c r="S13" s="82"/>
-      <c r="T13" s="83"/>
-      <c r="U13" s="84"/>
-    </row>
-    <row r="14" spans="1:21" ht="15.75">
+      <c r="S13" s="84"/>
+    </row>
+    <row r="14" spans="1:19" ht="15.75">
       <c r="A14" s="71" t="s">
         <v>25</v>
       </c>
@@ -2923,16 +2900,14 @@
       <c r="K14" s="79"/>
       <c r="L14" s="79"/>
       <c r="M14" s="80"/>
-      <c r="N14" s="66"/>
-      <c r="O14" s="66"/>
-      <c r="P14" s="81"/>
+      <c r="N14" s="81"/>
+      <c r="O14" s="82"/>
+      <c r="P14" s="83"/>
       <c r="Q14" s="82"/>
       <c r="R14" s="83"/>
-      <c r="S14" s="82"/>
-      <c r="T14" s="83"/>
-      <c r="U14" s="84"/>
-    </row>
-    <row r="15" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S14" s="84"/>
+    </row>
+    <row r="15" spans="1:19" ht="16.5" thickBot="1">
       <c r="A15" s="90" t="s">
         <v>27</v>
       </c>
@@ -2950,16 +2925,14 @@
       <c r="K15" s="79"/>
       <c r="L15" s="79"/>
       <c r="M15" s="80"/>
-      <c r="N15" s="66"/>
-      <c r="O15" s="66"/>
-      <c r="P15" s="94"/>
+      <c r="N15" s="94"/>
+      <c r="O15" s="95"/>
+      <c r="P15" s="96"/>
       <c r="Q15" s="95"/>
       <c r="R15" s="96"/>
-      <c r="S15" s="95"/>
-      <c r="T15" s="96"/>
-      <c r="U15" s="97"/>
-    </row>
-    <row r="16" spans="1:21" ht="16.5" thickTop="1">
+      <c r="S15" s="97"/>
+    </row>
+    <row r="16" spans="1:19" ht="16.5" thickTop="1">
       <c r="A16" s="90" t="s">
         <v>29</v>
       </c>
@@ -2977,18 +2950,16 @@
       <c r="K16" s="79"/>
       <c r="L16" s="79"/>
       <c r="M16" s="80"/>
-      <c r="N16" s="66"/>
-      <c r="O16" s="66"/>
-      <c r="P16" s="67" t="s">
+      <c r="N16" s="67" t="s">
         <v>20</v>
       </c>
+      <c r="O16" s="98"/>
+      <c r="P16" s="99"/>
       <c r="Q16" s="98"/>
       <c r="R16" s="99"/>
-      <c r="S16" s="98"/>
-      <c r="T16" s="99"/>
-      <c r="U16" s="100"/>
-    </row>
-    <row r="17" spans="1:21" ht="15.75">
+      <c r="S16" s="100"/>
+    </row>
+    <row r="17" spans="1:19" ht="15.75">
       <c r="A17" s="90" t="s">
         <v>31</v>
       </c>
@@ -3006,16 +2977,14 @@
       <c r="K17" s="79"/>
       <c r="L17" s="79"/>
       <c r="M17" s="80"/>
-      <c r="N17" s="66"/>
-      <c r="O17" s="66"/>
-      <c r="P17" s="101"/>
+      <c r="N17" s="101"/>
+      <c r="O17" s="82"/>
+      <c r="P17" s="83"/>
       <c r="Q17" s="82"/>
       <c r="R17" s="83"/>
-      <c r="S17" s="82"/>
-      <c r="T17" s="83"/>
-      <c r="U17" s="84"/>
-    </row>
-    <row r="18" spans="1:21" ht="15.75">
+      <c r="S17" s="84"/>
+    </row>
+    <row r="18" spans="1:19" ht="15.75">
       <c r="A18" s="71"/>
       <c r="B18" s="72"/>
       <c r="C18" s="72"/>
@@ -3031,16 +3000,14 @@
       <c r="K18" s="79"/>
       <c r="L18" s="79"/>
       <c r="M18" s="80"/>
-      <c r="N18" s="66"/>
-      <c r="O18" s="66"/>
-      <c r="P18" s="101"/>
+      <c r="N18" s="101"/>
+      <c r="O18" s="82"/>
+      <c r="P18" s="83"/>
       <c r="Q18" s="82"/>
       <c r="R18" s="83"/>
-      <c r="S18" s="82"/>
-      <c r="T18" s="83"/>
-      <c r="U18" s="84"/>
-    </row>
-    <row r="19" spans="1:21" ht="15.75">
+      <c r="S18" s="84"/>
+    </row>
+    <row r="19" spans="1:19" ht="15.75">
       <c r="A19" s="105"/>
       <c r="B19" s="106"/>
       <c r="C19" s="76"/>
@@ -3056,16 +3023,14 @@
       <c r="K19" s="79"/>
       <c r="L19" s="79"/>
       <c r="M19" s="80"/>
-      <c r="N19" s="66"/>
-      <c r="O19" s="66"/>
-      <c r="P19" s="101"/>
+      <c r="N19" s="101"/>
+      <c r="O19" s="82"/>
+      <c r="P19" s="83"/>
       <c r="Q19" s="82"/>
       <c r="R19" s="83"/>
-      <c r="S19" s="82"/>
-      <c r="T19" s="83"/>
-      <c r="U19" s="107"/>
-    </row>
-    <row r="20" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S19" s="107"/>
+    </row>
+    <row r="20" spans="1:19" ht="16.5" thickBot="1">
       <c r="A20" s="90"/>
       <c r="B20" s="91"/>
       <c r="C20" s="108"/>
@@ -3081,16 +3046,14 @@
       <c r="K20" s="111"/>
       <c r="L20" s="111"/>
       <c r="M20" s="112"/>
-      <c r="N20" s="113"/>
-      <c r="O20" s="113"/>
-      <c r="P20" s="114"/>
+      <c r="N20" s="114"/>
+      <c r="O20" s="95"/>
+      <c r="P20" s="96"/>
       <c r="Q20" s="95"/>
       <c r="R20" s="96"/>
-      <c r="S20" s="95"/>
-      <c r="T20" s="96"/>
-      <c r="U20" s="115"/>
-    </row>
-    <row r="21" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S20" s="115"/>
+    </row>
+    <row r="21" spans="1:19" ht="16.5" thickBot="1">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="108"/>
@@ -3106,16 +3069,14 @@
       <c r="K21" s="79"/>
       <c r="L21" s="79"/>
       <c r="M21" s="80"/>
-      <c r="N21" s="66"/>
-      <c r="O21" s="66"/>
-      <c r="P21" s="116"/>
+      <c r="N21" s="116"/>
+      <c r="O21" s="98"/>
+      <c r="P21" s="99"/>
       <c r="Q21" s="98"/>
       <c r="R21" s="99"/>
-      <c r="S21" s="98"/>
-      <c r="T21" s="99"/>
-      <c r="U21" s="100"/>
-    </row>
-    <row r="22" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S21" s="100"/>
+    </row>
+    <row r="22" spans="1:19" ht="16.5" thickBot="1">
       <c r="A22" s="90"/>
       <c r="B22" s="91"/>
       <c r="C22" s="108"/>
@@ -3129,16 +3090,14 @@
       <c r="K22" s="79"/>
       <c r="L22" s="79"/>
       <c r="M22" s="80"/>
-      <c r="N22" s="66"/>
-      <c r="O22" s="66"/>
-      <c r="P22" s="120"/>
+      <c r="N22" s="120"/>
+      <c r="O22" s="82"/>
+      <c r="P22" s="83"/>
       <c r="Q22" s="82"/>
       <c r="R22" s="83"/>
-      <c r="S22" s="82"/>
-      <c r="T22" s="83"/>
-      <c r="U22" s="84"/>
-    </row>
-    <row r="23" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S22" s="84"/>
+    </row>
+    <row r="23" spans="1:19" ht="16.5" thickBot="1">
       <c r="A23" s="121" t="s">
         <v>37</v>
       </c>
@@ -3156,16 +3115,14 @@
       <c r="K23" s="111"/>
       <c r="L23" s="111"/>
       <c r="M23" s="112"/>
-      <c r="N23" s="113"/>
-      <c r="O23" s="113"/>
-      <c r="P23" s="120"/>
+      <c r="N23" s="120"/>
+      <c r="O23" s="82"/>
+      <c r="P23" s="83"/>
       <c r="Q23" s="82"/>
       <c r="R23" s="83"/>
-      <c r="S23" s="82"/>
-      <c r="T23" s="83"/>
-      <c r="U23" s="127"/>
-    </row>
-    <row r="24" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S23" s="127"/>
+    </row>
+    <row r="24" spans="1:19" ht="16.5" thickBot="1">
       <c r="A24" s="128"/>
       <c r="B24" s="129"/>
       <c r="C24" s="129"/>
@@ -3181,16 +3138,14 @@
       <c r="K24" s="79"/>
       <c r="L24" s="79"/>
       <c r="M24" s="80"/>
-      <c r="N24" s="66"/>
-      <c r="O24" s="66"/>
-      <c r="P24" s="120"/>
+      <c r="N24" s="120"/>
+      <c r="O24" s="95"/>
+      <c r="P24" s="96"/>
       <c r="Q24" s="95"/>
       <c r="R24" s="96"/>
-      <c r="S24" s="95"/>
-      <c r="T24" s="96"/>
-      <c r="U24" s="97"/>
-    </row>
-    <row r="25" spans="1:21" ht="17.25" thickTop="1" thickBot="1">
+      <c r="S24" s="97"/>
+    </row>
+    <row r="25" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A25" s="134"/>
       <c r="B25" s="135"/>
       <c r="C25" s="135"/>
@@ -3206,16 +3161,14 @@
       <c r="K25" s="111"/>
       <c r="L25" s="111"/>
       <c r="M25" s="112"/>
-      <c r="N25" s="113"/>
-      <c r="O25" s="113"/>
-      <c r="P25" s="67"/>
+      <c r="N25" s="67"/>
+      <c r="O25" s="137"/>
+      <c r="P25" s="138"/>
       <c r="Q25" s="137"/>
       <c r="R25" s="138"/>
-      <c r="S25" s="137"/>
-      <c r="T25" s="138"/>
-      <c r="U25" s="139"/>
-    </row>
-    <row r="26" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S25" s="139"/>
+    </row>
+    <row r="26" spans="1:19" ht="16.5" thickBot="1">
       <c r="A26" s="140" t="s">
         <v>41</v>
       </c>
@@ -3233,16 +3186,14 @@
       <c r="K26" s="144"/>
       <c r="L26" s="144"/>
       <c r="M26" s="145"/>
-      <c r="N26" s="113"/>
-      <c r="O26" s="113"/>
-      <c r="P26" s="101"/>
+      <c r="N26" s="101"/>
+      <c r="O26" s="82"/>
+      <c r="P26" s="83"/>
       <c r="Q26" s="82"/>
       <c r="R26" s="83"/>
-      <c r="S26" s="82"/>
-      <c r="T26" s="83"/>
-      <c r="U26" s="146"/>
-    </row>
-    <row r="27" spans="1:21" ht="15.75">
+      <c r="S26" s="146"/>
+    </row>
+    <row r="27" spans="1:19" ht="15.75">
       <c r="A27" s="128"/>
       <c r="B27" s="129"/>
       <c r="C27" s="129"/>
@@ -3256,16 +3207,14 @@
       <c r="K27" s="79"/>
       <c r="L27" s="79"/>
       <c r="M27" s="80"/>
-      <c r="N27" s="66"/>
-      <c r="O27" s="66"/>
-      <c r="P27" s="101"/>
+      <c r="N27" s="101"/>
+      <c r="O27" s="82"/>
+      <c r="P27" s="83"/>
       <c r="Q27" s="82"/>
       <c r="R27" s="83"/>
-      <c r="S27" s="82"/>
-      <c r="T27" s="83"/>
-      <c r="U27" s="84"/>
-    </row>
-    <row r="28" spans="1:21" ht="15.75">
+      <c r="S27" s="84"/>
+    </row>
+    <row r="28" spans="1:19" ht="15.75">
       <c r="A28" s="134"/>
       <c r="B28" s="135"/>
       <c r="C28" s="135"/>
@@ -3281,16 +3230,14 @@
       <c r="K28" s="151"/>
       <c r="L28" s="151"/>
       <c r="M28" s="152"/>
-      <c r="N28" s="66"/>
-      <c r="O28" s="66"/>
-      <c r="P28" s="101"/>
+      <c r="N28" s="101"/>
+      <c r="O28" s="82"/>
+      <c r="P28" s="83"/>
       <c r="Q28" s="82"/>
       <c r="R28" s="83"/>
-      <c r="S28" s="82"/>
-      <c r="T28" s="83"/>
-      <c r="U28" s="107"/>
-    </row>
-    <row r="29" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S28" s="107"/>
+    </row>
+    <row r="29" spans="1:19" ht="16.5" thickBot="1">
       <c r="A29" s="153"/>
       <c r="B29" s="154"/>
       <c r="C29" s="154"/>
@@ -3306,16 +3253,14 @@
       <c r="K29" s="159"/>
       <c r="L29" s="159"/>
       <c r="M29" s="152"/>
-      <c r="N29" s="66"/>
-      <c r="O29" s="66"/>
-      <c r="P29" s="114"/>
-      <c r="Q29" s="82"/>
-      <c r="R29" s="83"/>
-      <c r="S29" s="160"/>
-      <c r="T29" s="161"/>
-      <c r="U29" s="162"/>
-    </row>
-    <row r="30" spans="1:21" ht="17.25" thickTop="1" thickBot="1">
+      <c r="N29" s="114"/>
+      <c r="O29" s="82"/>
+      <c r="P29" s="83"/>
+      <c r="Q29" s="160"/>
+      <c r="R29" s="161"/>
+      <c r="S29" s="162"/>
+    </row>
+    <row r="30" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A30" s="163" t="s">
         <v>45</v>
       </c>
@@ -3335,22 +3280,20 @@
       <c r="K30" s="164"/>
       <c r="L30" s="164"/>
       <c r="M30" s="165"/>
-      <c r="N30" s="170"/>
-      <c r="O30" s="170"/>
-      <c r="P30" s="171" t="s">
+      <c r="N30" s="171" t="s">
         <v>48</v>
       </c>
-      <c r="Q30" s="165"/>
-      <c r="R30" s="172" t="s">
+      <c r="O30" s="165"/>
+      <c r="P30" s="172" t="s">
         <v>49</v>
       </c>
-      <c r="S30" s="173"/>
-      <c r="T30" s="174" t="s">
+      <c r="Q30" s="173"/>
+      <c r="R30" s="174" t="s">
         <v>50</v>
       </c>
-      <c r="U30" s="175"/>
-    </row>
-    <row r="31" spans="1:21" ht="15.75">
+      <c r="S30" s="175"/>
+    </row>
+    <row r="31" spans="1:19" ht="15.75">
       <c r="A31" s="176" t="s">
         <v>51</v>
       </c>
@@ -3376,20 +3319,18 @@
       <c r="M31" s="187">
         <v>20</v>
       </c>
-      <c r="N31" s="188"/>
-      <c r="O31" s="188"/>
-      <c r="P31" s="189" t="s">
+      <c r="N31" s="189" t="s">
         <v>54</v>
       </c>
-      <c r="Q31" s="187">
+      <c r="O31" s="187">
         <v>500</v>
       </c>
+      <c r="P31" s="190"/>
+      <c r="Q31" s="191"/>
       <c r="R31" s="190"/>
-      <c r="S31" s="191"/>
-      <c r="T31" s="190"/>
-      <c r="U31" s="62"/>
-    </row>
-    <row r="32" spans="1:21" ht="15.75">
+      <c r="S31" s="62"/>
+    </row>
+    <row r="32" spans="1:19" ht="15.75">
       <c r="A32" s="192" t="s">
         <v>55</v>
       </c>
@@ -3407,16 +3348,14 @@
       <c r="K32" s="201"/>
       <c r="L32" s="106"/>
       <c r="M32" s="199"/>
-      <c r="N32" s="202"/>
-      <c r="O32" s="202"/>
-      <c r="P32" s="195"/>
-      <c r="Q32" s="199"/>
+      <c r="N32" s="195"/>
+      <c r="O32" s="199"/>
+      <c r="P32" s="200"/>
+      <c r="Q32" s="203"/>
       <c r="R32" s="200"/>
-      <c r="S32" s="203"/>
-      <c r="T32" s="200"/>
-      <c r="U32" s="77"/>
-    </row>
-    <row r="33" spans="1:21" ht="15.75">
+      <c r="S32" s="77"/>
+    </row>
+    <row r="33" spans="1:19" ht="15.75">
       <c r="A33" s="192" t="s">
         <v>57</v>
       </c>
@@ -3434,16 +3373,14 @@
       <c r="K33" s="201"/>
       <c r="L33" s="106"/>
       <c r="M33" s="199"/>
-      <c r="N33" s="202"/>
-      <c r="O33" s="202"/>
-      <c r="P33" s="195"/>
-      <c r="Q33" s="199"/>
+      <c r="N33" s="195"/>
+      <c r="O33" s="199"/>
+      <c r="P33" s="200"/>
+      <c r="Q33" s="203"/>
       <c r="R33" s="200"/>
-      <c r="S33" s="203"/>
-      <c r="T33" s="200"/>
-      <c r="U33" s="77"/>
-    </row>
-    <row r="34" spans="1:21" ht="15.75">
+      <c r="S33" s="77"/>
+    </row>
+    <row r="34" spans="1:19" ht="15.75">
       <c r="A34" s="192" t="s">
         <v>58</v>
       </c>
@@ -3461,16 +3398,14 @@
       <c r="K34" s="201"/>
       <c r="L34" s="106"/>
       <c r="M34" s="199"/>
-      <c r="N34" s="202"/>
-      <c r="O34" s="202"/>
-      <c r="P34" s="195"/>
-      <c r="Q34" s="199"/>
+      <c r="N34" s="195"/>
+      <c r="O34" s="199"/>
+      <c r="P34" s="200"/>
+      <c r="Q34" s="203"/>
       <c r="R34" s="200"/>
-      <c r="S34" s="203"/>
-      <c r="T34" s="200"/>
-      <c r="U34" s="77"/>
-    </row>
-    <row r="35" spans="1:21" ht="15.75">
+      <c r="S34" s="77"/>
+    </row>
+    <row r="35" spans="1:19" ht="15.75">
       <c r="A35" s="192" t="s">
         <v>59</v>
       </c>
@@ -3486,16 +3421,14 @@
       <c r="K35" s="201"/>
       <c r="L35" s="106"/>
       <c r="M35" s="199"/>
-      <c r="N35" s="202"/>
-      <c r="O35" s="202"/>
-      <c r="P35" s="195"/>
-      <c r="Q35" s="199"/>
+      <c r="N35" s="195"/>
+      <c r="O35" s="199"/>
+      <c r="P35" s="200"/>
+      <c r="Q35" s="203"/>
       <c r="R35" s="200"/>
-      <c r="S35" s="203"/>
-      <c r="T35" s="200"/>
-      <c r="U35" s="77"/>
-    </row>
-    <row r="36" spans="1:21" ht="16.5" thickBot="1">
+      <c r="S35" s="77"/>
+    </row>
+    <row r="36" spans="1:19" ht="16.5" thickBot="1">
       <c r="A36" s="105"/>
       <c r="B36" s="201"/>
       <c r="C36" s="106"/>
@@ -3509,16 +3442,14 @@
       <c r="K36" s="122"/>
       <c r="L36" s="206"/>
       <c r="M36" s="207"/>
-      <c r="N36" s="208"/>
-      <c r="O36" s="208"/>
-      <c r="P36" s="204"/>
-      <c r="Q36" s="207"/>
-      <c r="R36" s="205"/>
-      <c r="S36" s="209"/>
-      <c r="T36" s="200"/>
-      <c r="U36" s="77"/>
-    </row>
-    <row r="37" spans="1:21" ht="16.5" thickBot="1">
+      <c r="N36" s="204"/>
+      <c r="O36" s="207"/>
+      <c r="P36" s="205"/>
+      <c r="Q36" s="209"/>
+      <c r="R36" s="200"/>
+      <c r="S36" s="77"/>
+    </row>
+    <row r="37" spans="1:19" ht="16.5" thickBot="1">
       <c r="A37" s="210"/>
       <c r="B37" s="211"/>
       <c r="C37" s="211"/>
@@ -3532,20 +3463,18 @@
       <c r="K37" s="211"/>
       <c r="L37" s="211"/>
       <c r="M37" s="211"/>
-      <c r="N37" s="214"/>
-      <c r="O37" s="214"/>
-      <c r="P37" s="212"/>
+      <c r="N37" s="212"/>
+      <c r="O37" s="213"/>
+      <c r="P37" s="212" t="s">
+        <v>60</v>
+      </c>
       <c r="Q37" s="213"/>
       <c r="R37" s="212" t="s">
         <v>60</v>
       </c>
-      <c r="S37" s="213"/>
-      <c r="T37" s="212" t="s">
-        <v>60</v>
-      </c>
-      <c r="U37" s="215"/>
-    </row>
-    <row r="38" spans="1:21" ht="16.5" thickTop="1" thickBot="1">
+      <c r="S37" s="215"/>
+    </row>
+    <row r="38" spans="1:19" ht="16.5" thickTop="1" thickBot="1">
       <c r="A38" s="51"/>
       <c r="B38" s="51"/>
       <c r="C38" s="51"/>
@@ -3565,10 +3494,8 @@
       <c r="Q38" s="51"/>
       <c r="R38" s="51"/>
       <c r="S38" s="51"/>
-      <c r="T38" s="51"/>
-      <c r="U38" s="51"/>
-    </row>
-    <row r="39" spans="1:21">
+    </row>
+    <row r="39" spans="1:19">
       <c r="A39" s="2" t="s">
         <v>61</v>
       </c>
@@ -3588,16 +3515,14 @@
       <c r="M39" s="217"/>
       <c r="N39" s="217"/>
       <c r="O39" s="217"/>
-      <c r="P39" s="217"/>
-      <c r="Q39" s="217"/>
-      <c r="R39" s="218"/>
-      <c r="S39" s="219" t="s">
+      <c r="P39" s="218"/>
+      <c r="Q39" s="219" t="s">
         <v>63</v>
       </c>
-      <c r="T39" s="220"/>
-      <c r="U39" s="221"/>
-    </row>
-    <row r="40" spans="1:21" ht="15.75" thickBot="1">
+      <c r="R39" s="220"/>
+      <c r="S39" s="221"/>
+    </row>
+    <row r="40" spans="1:19" ht="15.75" thickBot="1">
       <c r="A40" s="14" t="s">
         <v>64</v>
       </c>
@@ -3615,137 +3540,135 @@
       <c r="M40" s="223"/>
       <c r="N40" s="223"/>
       <c r="O40" s="223"/>
-      <c r="P40" s="223"/>
-      <c r="Q40" s="223"/>
-      <c r="R40" s="224"/>
-      <c r="S40" s="225"/>
-      <c r="T40" s="226"/>
-      <c r="U40" s="227"/>
+      <c r="P40" s="224"/>
+      <c r="Q40" s="225"/>
+      <c r="R40" s="226"/>
+      <c r="S40" s="227"/>
     </row>
   </sheetData>
   <mergeCells count="169">
-    <mergeCell ref="D39:R40"/>
-    <mergeCell ref="S39:U40"/>
+    <mergeCell ref="D39:P40"/>
+    <mergeCell ref="Q39:S40"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="J37:M37"/>
+    <mergeCell ref="N37:O37"/>
     <mergeCell ref="P37:Q37"/>
     <mergeCell ref="R37:S37"/>
-    <mergeCell ref="T37:U37"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="E35:H35"/>
     <mergeCell ref="J35:L35"/>
+    <mergeCell ref="P35:Q35"/>
     <mergeCell ref="R35:S35"/>
-    <mergeCell ref="T35:U35"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="E36:H36"/>
     <mergeCell ref="J36:L36"/>
+    <mergeCell ref="P36:Q36"/>
     <mergeCell ref="R36:S36"/>
-    <mergeCell ref="T36:U36"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="E33:H33"/>
     <mergeCell ref="J33:L33"/>
+    <mergeCell ref="P33:Q33"/>
     <mergeCell ref="R33:S33"/>
-    <mergeCell ref="T33:U33"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="E34:H34"/>
     <mergeCell ref="J34:L34"/>
+    <mergeCell ref="P34:Q34"/>
     <mergeCell ref="R34:S34"/>
-    <mergeCell ref="T34:U34"/>
-    <mergeCell ref="T31:U31"/>
+    <mergeCell ref="R31:S31"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="E32:H32"/>
     <mergeCell ref="J32:L32"/>
+    <mergeCell ref="P32:Q32"/>
     <mergeCell ref="R32:S32"/>
-    <mergeCell ref="T32:U32"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="J30:M30"/>
+    <mergeCell ref="N30:O30"/>
     <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="R30:S30"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="E31:H31"/>
     <mergeCell ref="J31:L31"/>
-    <mergeCell ref="R31:S31"/>
-    <mergeCell ref="S27:T27"/>
+    <mergeCell ref="P31:Q31"/>
+    <mergeCell ref="Q27:R27"/>
     <mergeCell ref="E28:G28"/>
     <mergeCell ref="H28:I28"/>
+    <mergeCell ref="O28:P28"/>
     <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="S28:T28"/>
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="H29:I29"/>
+    <mergeCell ref="O29:P29"/>
     <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="S29:T29"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="C27:C29"/>
     <mergeCell ref="D27:D29"/>
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="H27:I27"/>
-    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="O27:P27"/>
     <mergeCell ref="H25:I25"/>
-    <mergeCell ref="P25:P29"/>
+    <mergeCell ref="N25:N29"/>
+    <mergeCell ref="O25:P25"/>
     <mergeCell ref="Q25:R25"/>
-    <mergeCell ref="S25:T25"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="E26:G26"/>
     <mergeCell ref="H26:I26"/>
+    <mergeCell ref="O26:P26"/>
     <mergeCell ref="Q26:R26"/>
-    <mergeCell ref="S26:T26"/>
     <mergeCell ref="A27:A29"/>
-    <mergeCell ref="S23:T23"/>
+    <mergeCell ref="Q23:R23"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="C24:C25"/>
     <mergeCell ref="D24:D25"/>
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="H24:I24"/>
+    <mergeCell ref="O24:P24"/>
     <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="S24:T24"/>
     <mergeCell ref="E25:G25"/>
-    <mergeCell ref="S21:T21"/>
+    <mergeCell ref="Q21:R21"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="E22:G22"/>
     <mergeCell ref="H22:I22"/>
+    <mergeCell ref="O22:P22"/>
     <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="S22:T22"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="E21:G21"/>
     <mergeCell ref="H21:I21"/>
-    <mergeCell ref="P21:P24"/>
-    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="N21:N24"/>
+    <mergeCell ref="O21:P21"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:I23"/>
-    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="O23:P23"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="E20:G20"/>
     <mergeCell ref="H20:I20"/>
+    <mergeCell ref="O20:P20"/>
     <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="S20:T20"/>
+    <mergeCell ref="O18:P18"/>
     <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="S18:T18"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="H19:I19"/>
+    <mergeCell ref="O19:P19"/>
     <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="S19:T19"/>
-    <mergeCell ref="S16:T16"/>
+    <mergeCell ref="Q16:R16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="H17:I17"/>
+    <mergeCell ref="O17:P17"/>
     <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="S17:T17"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="E16:G16"/>
     <mergeCell ref="H16:I16"/>
-    <mergeCell ref="P16:P20"/>
-    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="N16:N20"/>
+    <mergeCell ref="O16:P16"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="E18:G18"/>
@@ -3754,45 +3677,45 @@
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:I15"/>
+    <mergeCell ref="O15:P15"/>
     <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="S13:T13"/>
+    <mergeCell ref="Q13:R13"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="H14:I14"/>
+    <mergeCell ref="O14:P14"/>
     <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="S14:T14"/>
-    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="Q11:R11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="E12:G12"/>
     <mergeCell ref="H12:I12"/>
+    <mergeCell ref="O12:P12"/>
     <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="S12:T12"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="H11:I11"/>
-    <mergeCell ref="P11:P15"/>
-    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="N11:N15"/>
+    <mergeCell ref="O11:P11"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="H13:I13"/>
-    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="O13:P13"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="C9:I9"/>
     <mergeCell ref="J9:M9"/>
-    <mergeCell ref="P9:U9"/>
+    <mergeCell ref="N9:S9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="E10:I10"/>
+    <mergeCell ref="O10:P10"/>
     <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="S10:T10"/>
-    <mergeCell ref="E2:U3"/>
-    <mergeCell ref="E4:U5"/>
-    <mergeCell ref="A7:U7"/>
+    <mergeCell ref="E2:S3"/>
+    <mergeCell ref="E4:S5"/>
+    <mergeCell ref="A7:S7"/>
     <mergeCell ref="A8:I8"/>
     <mergeCell ref="J8:M8"/>
-    <mergeCell ref="P8:U8"/>
+    <mergeCell ref="N8:S8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>